<commit_message>
feat: complete Google Sheets sync integration and Code.gs backend
</commit_message>
<xml_diff>
--- a/sheets/pycrm_database.xlsx
+++ b/sheets/pycrm_database.xlsx
@@ -662,7 +662,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -702,16 +702,89 @@
         <v>candidateId</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>reg_20260522_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>new.candidate@email.com</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Ananya Rao</v>
+      </c>
+      <c r="D2" t="str">
+        <v>new.candidate@email.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>+91 90000 11111</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1999-09-15</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Velachery, Chennai</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Python Core</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Chennai</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2025-03-05T10:00:00Z</v>
+      </c>
+      <c r="K2" t="str">
+        <v>pending-import</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>reg_20260522_002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>lead.candidate@email.com</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Karthik Menon</v>
+      </c>
+      <c r="D3" t="str">
+        <v>lead.candidate@email.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>+91 90000 22222</v>
+      </c>
+      <c r="F3" t="str">
+        <v>1998-03-12</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Whitefield, Bangalore</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Full Stack</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Bangalore</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2025-03-06T10:00:00Z</v>
+      </c>
+      <c r="K3" t="str">
+        <v>candidate-created</v>
+      </c>
+      <c r="L3" t="str">
+        <v>c7</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -760,16 +833,63 @@
         <v>reviewStatus</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>bgv_20260522_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Rahul Sharma</v>
+      </c>
+      <c r="D2" t="str">
+        <v>rahul.sharma@email.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>+91 98765 43210</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1234 5678 9012</v>
+      </c>
+      <c r="G2" t="str">
+        <v>42, MG Road, Bangalore, Karnataka 560001</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Anita Sharma +91 90000 33333</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="str">
+        <v>2025-01-20T10:00:00Z</v>
+      </c>
+      <c r="O2" t="str">
+        <v>in-review</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -791,9 +911,49 @@
         <v>duration</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>bgv_20260522_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TCS</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Software Engineer</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2020-2022</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>bgv_20260522_001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Senior Developer</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2022-2024</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1145,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1172,7 +1332,7 @@
         <v>Displayed on public forms and settings</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-01-01</v>
+        <v>2026-06-03T13:46:30.314Z</v>
       </c>
     </row>
     <row r="3">
@@ -1186,26 +1346,54 @@
         <v>BGV team mail id used by dispatch flow</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-01-01</v>
+        <v>2026-06-03T13:46:30.314Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>gasWebAppUrl</v>
+      </c>
+      <c r="B4" t="str">
+        <v>https://script.googleusercontent.com/macros/echo?user_content_key=AUkAhnRExLRbGOzooffwsfYhe8LXEJuXYC5wjqJNKC_L4ZDOfnin-lrbqGALCnKP9dnUmJ-ZvXNfW39mgkhdEGh-Yec78RjBnBmIxudXCuP7vG95x7AyT13OjP5aPvuZDqvRmf-ESo4G1I9-JyzIkvEPe9ES2c12bUb7Eg1k6tCihFeGoTlYhDX0Uq0w-mt1od_c0ujilFnLAnsszx9GdQji8DXy50FdtEodDJ-gy3pXzn3pSwz3ri0Pgb1ibigIn4kLQ8h9a2wv5swe38setFuOT_Ok8vygCA&amp;lib=MbHEaKX0aWK7LN2vKPMZcvTE2IrMUDdkp</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Required for sending form links without backend server</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-06-03T13:46:30.314Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>themeMode</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v>command</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C5" t="str">
         <v>UI preference only; app may persist this locally</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D5" t="str">
         <v>2025-01-01</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>hrCCEmail</v>
+      </c>
+      <c r="B6" t="str">
+        <v>hr@pythonhr.com</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-06-03T13:46:30.314Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1236,7 +1424,7 @@
         <v>Candidate Master Sheet</v>
       </c>
       <c r="C2" t="str">
-        <v>https://forms.gle/7MgUZ5zpj5by5EK37</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v>Primary candidate profile and status data</v>
@@ -1250,7 +1438,7 @@
         <v>Registration Responses Sheet</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>https://docs.google.com/forms/d/1jReIE9nZ-LlDePPCm6zYJfItyqpSI9wkrBtM5ke7vkQ/prefill</v>
       </c>
       <c r="D3" t="str">
         <v>New registration form submissions</v>
@@ -1321,7 +1509,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:R5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1379,16 +1567,213 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Rahul Sharma</v>
+      </c>
+      <c r="C2" t="str">
+        <v>rahul.sharma@email.com</v>
+      </c>
+      <c r="D2" t="str">
+        <v>+91 98765 43210</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Batch 4</v>
+      </c>
+      <c r="F2" t="str">
+        <v>1995-03-15</v>
+      </c>
+      <c r="G2" t="str">
+        <v>42, MG Road, Bangalore, Karnataka 560001</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Bangalore</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Full Stack</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2025-01-10</v>
+      </c>
+      <c r="K2" t="str">
+        <v>active</v>
+      </c>
+      <c r="L2" t="str">
+        <v>pending</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>2025-01-10</v>
+      </c>
+      <c r="R2" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Priya Patel</v>
+      </c>
+      <c r="C3" t="str">
+        <v>priya.patel@email.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>+91 87654 32109</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Batch 5</v>
+      </c>
+      <c r="F3" t="str">
+        <v>1997-08-22</v>
+      </c>
+      <c r="G3" t="str">
+        <v>15, Park Street, Mumbai, Maharashtra 400001</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Online</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Python Core</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2025-02-05</v>
+      </c>
+      <c r="K3" t="str">
+        <v>active</v>
+      </c>
+      <c r="L3" t="str">
+        <v>in-review</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>2025-02-05</v>
+      </c>
+      <c r="R3" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Amit Kumar</v>
+      </c>
+      <c r="C4" t="str">
+        <v>amit.kumar@email.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>+91 76543 21098</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Batch 3</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1993-11-05</v>
+      </c>
+      <c r="G4" t="str">
+        <v>78, Salt Lake, Kolkata, West Bengal 700091</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Chennai</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Python Core</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2024-12-01</v>
+      </c>
+      <c r="K4" t="str">
+        <v>active</v>
+      </c>
+      <c r="L4" t="str">
+        <v>cleared</v>
+      </c>
+      <c r="M4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Google India</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>2024-12-01</v>
+      </c>
+      <c r="R4" t="str">
+        <v>2025-01-15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Sneha Reddy</v>
+      </c>
+      <c r="C5" t="str">
+        <v>sneha.reddy@email.com</v>
+      </c>
+      <c r="D5" t="str">
+        <v>+91 65432 10987</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Batch 6</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1996-06-18</v>
+      </c>
+      <c r="G5" t="str">
+        <v>33, Jubilee Hills, Hyderabad, Telangana 500033</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Bangalore</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Full Stack</v>
+      </c>
+      <c r="J5" t="str">
+        <v>2025-03-01</v>
+      </c>
+      <c r="K5" t="str">
+        <v>active</v>
+      </c>
+      <c r="L5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="str">
+        <v>form-pending</v>
+      </c>
+      <c r="P5" t="str">
+        <v>2025-03-01</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>2025-03-01</v>
+      </c>
+      <c r="R5" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1410,16 +1795,416 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>offerLetter</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Offer Letter</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>appraisals</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Appraisals</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>payslips</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Payslips</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>relievingLetter</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Relieving Letter</v>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B6" t="str">
+        <v>counterOffer</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Counter Offer</v>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B7" t="str">
+        <v>offerLetter</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Offer Letter</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B8" t="str">
+        <v>appraisals</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Appraisals</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B9" t="str">
+        <v>payslips</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Payslips</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B10" t="str">
+        <v>relievingLetter</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Relieving Letter</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B11" t="str">
+        <v>counterOffer</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Counter Offer</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B12" t="str">
+        <v>offerLetter</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Offer Letter</v>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B13" t="str">
+        <v>appraisals</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Appraisals</v>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B14" t="str">
+        <v>payslips</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Payslips</v>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B15" t="str">
+        <v>relievingLetter</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Relieving Letter</v>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B16" t="str">
+        <v>counterOffer</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Counter Offer</v>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B17" t="str">
+        <v>offerLetter</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Offer Letter</v>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B18" t="str">
+        <v>appraisals</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Appraisals</v>
+      </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B19" t="str">
+        <v>payslips</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Payslips</v>
+      </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B20" t="str">
+        <v>relievingLetter</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Relieving Letter</v>
+      </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B21" t="str">
+        <v>counterOffer</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Counter Offer</v>
+      </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1447,16 +2232,176 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>emp_c1_1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TCS</v>
+      </c>
+      <c r="F2" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>emp_c1_2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Infosys</v>
+      </c>
+      <c r="F3" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>emp_c2_1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>c2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Cognizant</v>
+      </c>
+      <c r="F4" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>emp_c2_2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>c2</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Wipro</v>
+      </c>
+      <c r="F5" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>emp_c3_1</v>
+      </c>
+      <c r="B6" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C6" t="str">
+        <v>HCL</v>
+      </c>
+      <c r="F6" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>emp_c3_2</v>
+      </c>
+      <c r="B7" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Tech Mahindra</v>
+      </c>
+      <c r="F7" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>emp_c3_3</v>
+      </c>
+      <c r="B8" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Accenture</v>
+      </c>
+      <c r="F8" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>emp_c4_1</v>
+      </c>
+      <c r="B9" t="str">
+        <v>c4</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Capgemini</v>
+      </c>
+      <c r="F9" t="str">
+        <v>profile</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1487,16 +2432,480 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>registration</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Registration Fee</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>course</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Course Fee</v>
+      </c>
+      <c r="D3">
+        <v>30000</v>
+      </c>
+      <c r="E3">
+        <v>-2000</v>
+      </c>
+      <c r="F3">
+        <v>25000</v>
+      </c>
+      <c r="G3">
+        <v>28000</v>
+      </c>
+      <c r="H3">
+        <v>3000</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>document</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Document Fee</v>
+      </c>
+      <c r="D4">
+        <v>25000</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>25000</v>
+      </c>
+      <c r="H4">
+        <v>25000</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>c1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>placement</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Placement Payment</v>
+      </c>
+      <c r="D5">
+        <v>100000</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>100000</v>
+      </c>
+      <c r="H5">
+        <v>100000</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2025-01-10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B6" t="str">
+        <v>registration</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Registration Fee</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B7" t="str">
+        <v>course</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Course Fee</v>
+      </c>
+      <c r="D7">
+        <v>30000</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>10000</v>
+      </c>
+      <c r="G7">
+        <v>30000</v>
+      </c>
+      <c r="H7">
+        <v>20000</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B8" t="str">
+        <v>document</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Document Fee</v>
+      </c>
+      <c r="D8">
+        <v>25000</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>5000</v>
+      </c>
+      <c r="G8">
+        <v>25000</v>
+      </c>
+      <c r="H8">
+        <v>20000</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B9" t="str">
+        <v>placement</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Placement Payment</v>
+      </c>
+      <c r="D9">
+        <v>100000</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>100000</v>
+      </c>
+      <c r="H9">
+        <v>100000</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2025-02-05</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B10" t="str">
+        <v>registration</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Registration Fee</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B11" t="str">
+        <v>course</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Course Fee</v>
+      </c>
+      <c r="D11">
+        <v>30000</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>30000</v>
+      </c>
+      <c r="G11">
+        <v>30000</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B12" t="str">
+        <v>document</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Document Fee</v>
+      </c>
+      <c r="D12">
+        <v>25000</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>25000</v>
+      </c>
+      <c r="G12">
+        <v>25000</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>c3</v>
+      </c>
+      <c r="B13" t="str">
+        <v>placement</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Placement Payment</v>
+      </c>
+      <c r="D13">
+        <v>100000</v>
+      </c>
+      <c r="E13">
+        <v>-10000</v>
+      </c>
+      <c r="F13">
+        <v>90000</v>
+      </c>
+      <c r="G13">
+        <v>90000</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B14" t="str">
+        <v>registration</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Registration Fee</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B15" t="str">
+        <v>course</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Course Fee</v>
+      </c>
+      <c r="D15">
+        <v>30000</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>30000</v>
+      </c>
+      <c r="H15">
+        <v>30000</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B16" t="str">
+        <v>document</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Document Fee</v>
+      </c>
+      <c r="D16">
+        <v>25000</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>25000</v>
+      </c>
+      <c r="H16">
+        <v>25000</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B17" t="str">
+        <v>placement</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Placement Payment</v>
+      </c>
+      <c r="D17">
+        <v>100000</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>100000</v>
+      </c>
+      <c r="H17">
+        <v>100000</v>
+      </c>
+      <c r="I17" t="str">
+        <v>2025-03-01</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1524,16 +2933,68 @@
         <v>userStamp</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>adj_c1_course_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>course</v>
+      </c>
+      <c r="D2">
+        <v>-2000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Corporate Waiver</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Branch Manager approved early-bird corporate waiver</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-01-10T10:30:00Z</v>
+      </c>
+      <c r="H2" t="str">
+        <v>HR-A</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>adj_c3_placement_001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C3" t="str">
+        <v>placement</v>
+      </c>
+      <c r="D3">
+        <v>-10000</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Placement Partner Credit</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Referral credit approved by placements team</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-01-15T09:15:00Z</v>
+      </c>
+      <c r="H3" t="str">
+        <v>HR-B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1561,16 +3022,172 @@
         <v>userStamp</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>pay_c1_course_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>course</v>
+      </c>
+      <c r="D2">
+        <v>25000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>TXN-C1-COURSE-001</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Paid via GPay - Batch 4</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-01-15T14:20:00Z</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Python HR</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>pay_c2_course_001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>c2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>course</v>
+      </c>
+      <c r="D3">
+        <v>10000</v>
+      </c>
+      <c r="E3" t="str">
+        <v>TXN-C2-COURSE-001</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Initial course payment</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-02-10T10:00:00Z</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Python HR</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>pay_c2_document_001</v>
+      </c>
+      <c r="B4" t="str">
+        <v>c2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>document</v>
+      </c>
+      <c r="D4">
+        <v>5000</v>
+      </c>
+      <c r="E4" t="str">
+        <v>TXN-C2-DOC-001</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Document fee part payment</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-02-15T10:00:00Z</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Python HR</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>pay_c3_course_001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C5" t="str">
+        <v>course</v>
+      </c>
+      <c r="D5">
+        <v>30000</v>
+      </c>
+      <c r="E5" t="str">
+        <v>TXN-C3-COURSE-001</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Course fee paid in full</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2024-12-10T10:00:00Z</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Python HR</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>pay_c3_document_001</v>
+      </c>
+      <c r="B6" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C6" t="str">
+        <v>document</v>
+      </c>
+      <c r="D6">
+        <v>25000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>TXN-C3-DOC-001</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Document fee paid in full</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2024-12-15T10:00:00Z</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Python HR</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>pay_c3_placement_001</v>
+      </c>
+      <c r="B7" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C7" t="str">
+        <v>placement</v>
+      </c>
+      <c r="D7">
+        <v>90000</v>
+      </c>
+      <c r="E7" t="str">
+        <v>TXN-C3-PLACE-001</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Placement payment after waiver</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2025-03-10T10:00:00Z</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Python HR</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1595,16 +3212,76 @@
         <v>timestamp</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>c4</v>
+      </c>
+      <c r="B2" t="str">
+        <v>form-pending</v>
+      </c>
+      <c r="C2" t="str">
+        <v>new-registration</v>
+      </c>
+      <c r="D2" t="str">
+        <v>sneha.reddy@email.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Sneha Reddy</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-03-01T10:00:00Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>bgv-submitted</v>
+      </c>
+      <c r="C3" t="str">
+        <v>bgv-form</v>
+      </c>
+      <c r="D3" t="str">
+        <v>priya.patel@email.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Priya Patel</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-02-05T10:00:00Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>tc_20260522_001</v>
+      </c>
+      <c r="B4" t="str">
+        <v>contacts-sent</v>
+      </c>
+      <c r="C4" t="str">
+        <v>contact-mail</v>
+      </c>
+      <c r="D4" t="str">
+        <v>lead.candidate@email.com</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-03-02T10:00:00Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1629,9 +3306,98 @@
         <v>timestamp</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>l1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>structural</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Applied discount: Corporate Waiver (-Rs.2,000)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Branch Manager approved early-bird corporate waiver</v>
+      </c>
+      <c r="F2" t="str">
+        <v>HR-A</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-01-10T10:30:00Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>l2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>c1</v>
+      </c>
+      <c r="C3" t="str">
+        <v>financial</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Payment received: Rs.25,000 for Course Fee</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Paid via GPay - Batch 4</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Python HR</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-01-15T14:20:00Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>l3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>c2</v>
+      </c>
+      <c r="C4" t="str">
+        <v>bgv</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BGV request dispatched to team</v>
+      </c>
+      <c r="F4" t="str">
+        <v>HR-A</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-02-05T10:00:00Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>l4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>c3</v>
+      </c>
+      <c r="C5" t="str">
+        <v>financial</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Python HR logged a payment of Rs.90,000 for Placement Payment. (Ref: TXN-C3-PLACE-001)</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Placement payment after waiver</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Python HR</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2025-03-10T10:00:00Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor CRM syncing pipeline, implement strict FullName mapping, and clear frontend mock data
</commit_message>
<xml_diff>
--- a/sheets/pycrm_database.xlsx
+++ b/sheets/pycrm_database.xlsx
@@ -1332,7 +1332,7 @@
         <v>Displayed on public forms and settings</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-06-03T13:46:30.314Z</v>
+        <v>2026-06-07T15:45:24.913Z</v>
       </c>
     </row>
     <row r="3">
@@ -1346,7 +1346,7 @@
         <v>BGV team mail id used by dispatch flow</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-06-03T13:46:30.314Z</v>
+        <v>2026-06-07T15:45:24.913Z</v>
       </c>
     </row>
     <row r="4">
@@ -1354,13 +1354,13 @@
         <v>gasWebAppUrl</v>
       </c>
       <c r="B4" t="str">
-        <v>https://script.googleusercontent.com/macros/echo?user_content_key=AUkAhnRExLRbGOzooffwsfYhe8LXEJuXYC5wjqJNKC_L4ZDOfnin-lrbqGALCnKP9dnUmJ-ZvXNfW39mgkhdEGh-Yec78RjBnBmIxudXCuP7vG95x7AyT13OjP5aPvuZDqvRmf-ESo4G1I9-JyzIkvEPe9ES2c12bUb7Eg1k6tCihFeGoTlYhDX0Uq0w-mt1od_c0ujilFnLAnsszx9GdQji8DXy50FdtEodDJ-gy3pXzn3pSwz3ri0Pgb1ibigIn4kLQ8h9a2wv5swe38setFuOT_Ok8vygCA&amp;lib=MbHEaKX0aWK7LN2vKPMZcvTE2IrMUDdkp</v>
+        <v>https://script.googleusercontent.com/macros/echo?user_content_key=AUkAhnQkrjHTd8kmJx6xzX5Rh3OGQSyy2-kOliEFFTHMTRmIXC1EqjZ6yFZ70qyqYMQYER6hy0wVbFRZtJeUZx49eoLBNzrL0dO4lkU5bmUOL_--_D0YNNTga6mq7M7zcZYfdaKe3wvQUy6gi4_XZMyG2qX-UHO4Zhy_Qr5vogg1DreNI59x6yv5Ohux2xBwaic4IBGUSnMmhLwkwTEOvDnFMGqNnyDnJUkbems1UV47xxQUuU1V0y33c1kLj867TFDP3AmCgOau3g0Jm-yzUYJqMzL7NpPAIw&amp;lib=Mj9GlV-mn6XtaOTKXe6iIboeeCcJJxTZN</v>
       </c>
       <c r="C4" t="str">
         <v>Required for sending form links without backend server</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-06-03T13:46:30.314Z</v>
+        <v>2026-06-07T15:45:24.913Z</v>
       </c>
     </row>
     <row r="5">
@@ -1388,7 +1388,7 @@
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>2026-06-03T13:46:30.314Z</v>
+        <v>2026-06-07T15:45:24.913Z</v>
       </c>
     </row>
   </sheetData>
@@ -1400,7 +1400,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1438,7 +1438,7 @@
         <v>Registration Responses Sheet</v>
       </c>
       <c r="C3" t="str">
-        <v>https://docs.google.com/forms/d/1jReIE9nZ-LlDePPCm6zYJfItyqpSI9wkrBtM5ke7vkQ/prefill</v>
+        <v/>
       </c>
       <c r="D3" t="str">
         <v>New registration form submissions</v>
@@ -1500,9 +1500,23 @@
         <v>Dropdowns, branches, and app configuration</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>registrationForm</v>
+      </c>
+      <c r="B8" t="str">
+        <v>registrationForm</v>
+      </c>
+      <c r="C8" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHboeBmumpOIhfagPmkqJM0MTZlcCNZGsWTd2KIyrOISt2BQ/viewform?usp=dialog</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add README and fix Settings page bug
</commit_message>
<xml_diff>
--- a/sheets/pycrm_database.xlsx
+++ b/sheets/pycrm_database.xlsx
@@ -1305,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1332,7 +1332,7 @@
         <v>Displayed on public forms and settings</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-06-09T17:16:52.701Z</v>
+        <v>2026-06-09T17:43:20.369Z</v>
       </c>
     </row>
     <row r="3">
@@ -1346,7 +1346,7 @@
         <v>BGV team mail id used by dispatch flow</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-06-09T17:16:52.701Z</v>
+        <v>2026-06-09T17:43:20.369Z</v>
       </c>
     </row>
     <row r="4">
@@ -1360,7 +1360,7 @@
         <v>Required for sending form links without backend server</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-06-09T17:16:52.701Z</v>
+        <v>2026-06-09T17:43:20.369Z</v>
       </c>
     </row>
     <row r="5">
@@ -1388,12 +1388,40 @@
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>2026-06-09T17:16:52.701Z</v>
+        <v>2026-06-09T17:43:20.369Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>courses</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Python Core,Full Stack,Data Science,Machine Learning,Web Development,Other</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-06-09T17:43:20.369Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>branches</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Chennai,Bangalore,Online</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-06-09T17:43:20.369Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: financial persistence, adjustment delete sync, and performance optimizations
- Fixed adjustment deletion synchronization issue where old adjustments returned after refresh due to case-mismatched pipelineType duplicate appending.
- Hardened adjustment calculations (Math.abs(Number(a.amount) || 0)) to handle legacy records safely without throwing NaN.
- Fixed race condition in CandidateProfile.tsx preventing fast payments from saving.
- Added strict mapping for Candidate Profile update headers to prevent duplicate columns in sheets.
- Added optimistic UI updates for payments and caching in the store for better responsiveness.
</commit_message>
<xml_diff>
--- a/sheets/pycrm_database.xlsx
+++ b/sheets/pycrm_database.xlsx
@@ -1332,7 +1332,7 @@
         <v>Displayed on public forms and settings</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-06-25T02:51:04.174Z</v>
+        <v>2026-06-25T20:17:05.876Z</v>
       </c>
     </row>
     <row r="3">
@@ -1346,7 +1346,7 @@
         <v>BGV team mail id used by dispatch flow</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-06-25T02:51:04.174Z</v>
+        <v>2026-06-25T20:17:05.876Z</v>
       </c>
     </row>
     <row r="4">
@@ -1360,7 +1360,7 @@
         <v>Required for sending form links without backend server</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-06-25T02:51:04.174Z</v>
+        <v>2026-06-25T20:17:05.876Z</v>
       </c>
     </row>
     <row r="5">
@@ -1388,7 +1388,7 @@
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>2026-06-25T02:51:04.174Z</v>
+        <v>2026-06-25T20:17:05.876Z</v>
       </c>
     </row>
     <row r="7">
@@ -1396,13 +1396,13 @@
         <v>courses</v>
       </c>
       <c r="B7" t="str">
-        <v>Python Fullstack,Python Advance,Snowflake / Data Analytics,Javascript React JS,Gen AI,AWS</v>
+        <v>Other,Python Fullstack,Python Advance,Snowflake/ Data Analytics,Javascript React js,Gen AI,Aws</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" t="str">
-        <v>2026-06-25T02:51:04.174Z</v>
+        <v>2026-06-25T20:17:05.876Z</v>
       </c>
     </row>
     <row r="8">
@@ -1410,13 +1410,13 @@
         <v>branches</v>
       </c>
       <c r="B8" t="str">
-        <v>Chennai,Madurai,Coimbatore,Salem,Tirunelveli,Trichy,Pondicherry,Bangalore</v>
+        <v>Chennai,Bangalore,Madurai,Coimbatore,Salem,Tirunelveli,Trichy,Pondicherry</v>
       </c>
       <c r="C8" t="str">
         <v/>
       </c>
       <c r="D8" t="str">
-        <v>2026-06-25T02:51:04.174Z</v>
+        <v>2026-06-25T20:17:05.876Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>